<commit_message>
adapted split violine plots
</commit_message>
<xml_diff>
--- a/similarity_t_tests/t_test_results.xlsx
+++ b/similarity_t_tests/t_test_results.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,42 +431,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>column</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>mean_orthologs</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>mean_swissprot</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>t_stat</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>p_value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>significant_0.05</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>n_orthologs</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>n_swissprot</t>
         </is>
@@ -467,22 +479,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.3929</v>
+        <v>4.3651</v>
       </c>
       <c r="C2" t="n">
         <v>3.0833</v>
       </c>
       <c r="D2" t="n">
-        <v>5.2518</v>
+        <v>5.2211</v>
       </c>
       <c r="E2" t="n">
-        <v>6e-06</v>
+        <v>7e-06</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H2" t="n">
         <v>24</v>
@@ -495,22 +507,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0558</v>
+        <v>0.0599</v>
       </c>
       <c r="C3" t="n">
         <v>0.0982</v>
       </c>
       <c r="D3" t="n">
-        <v>-4.219</v>
+        <v>-3.7479</v>
       </c>
       <c r="E3" t="n">
-        <v>0.000247</v>
+        <v>0.000789</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H3" t="n">
         <v>24</v>
@@ -519,26 +531,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>median_plddt</t>
+          <t>avg_plddt</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9736</v>
+        <v>0.95</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9597</v>
+        <v>0.9232</v>
       </c>
       <c r="D4" t="n">
-        <v>3.8535</v>
+        <v>3.0331</v>
       </c>
       <c r="E4" t="n">
-        <v>0.000541</v>
+        <v>0.004437</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H4" t="n">
         <v>24</v>
@@ -547,26 +559,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>avg_plddt</t>
+          <t>std_plddt_bs</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9549</v>
+        <v>0.0381</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9232</v>
+        <v>0.0766</v>
       </c>
       <c r="D5" t="n">
-        <v>3.8635</v>
+        <v>-2.9859</v>
       </c>
       <c r="E5" t="n">
-        <v>0.000613</v>
+        <v>0.005885</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H5" t="n">
         <v>24</v>
@@ -575,26 +587,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>median_plddt_bs</t>
+          <t>p10_plddt</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9757</v>
+        <v>0.8934</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9627</v>
+        <v>0.8094</v>
       </c>
       <c r="D6" t="n">
-        <v>3.4124</v>
+        <v>2.8747</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001826</v>
+        <v>0.007471</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H6" t="n">
         <v>24</v>
@@ -603,26 +615,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>avg_plddt_bs</t>
+          <t>tm_score</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9623</v>
+        <v>0.8383</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9321</v>
+        <v>0.8046</v>
       </c>
       <c r="D7" t="n">
-        <v>3.3937</v>
+        <v>2.8967</v>
       </c>
       <c r="E7" t="n">
-        <v>0.00217</v>
+        <v>0.007548</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H7" t="n">
         <v>24</v>
@@ -631,26 +643,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>p10_plddt</t>
+          <t>avg_plddt_bs</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9039</v>
+        <v>0.9584</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8094</v>
+        <v>0.9321</v>
       </c>
       <c r="D8" t="n">
-        <v>3.3208</v>
+        <v>2.7864</v>
       </c>
       <c r="E8" t="n">
-        <v>0.002634</v>
+        <v>0.008723</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H8" t="n">
         <v>24</v>
@@ -659,26 +671,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>std_plddt_bs</t>
+          <t>p10_plddt_bs</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0353</v>
+        <v>0.9126</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0766</v>
+        <v>0.8088</v>
       </c>
       <c r="D9" t="n">
-        <v>-3.255</v>
+        <v>2.8309</v>
       </c>
       <c r="E9" t="n">
-        <v>0.003156</v>
+        <v>0.008770999999999999</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H9" t="n">
         <v>24</v>
@@ -687,26 +699,26 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>p10_plddt_bs</t>
+          <t>cavity_n_points</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9222</v>
+        <v>2433.3968</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8088</v>
+        <v>2925.7083</v>
       </c>
       <c r="D10" t="n">
-        <v>3.1607</v>
+        <v>-2.5829</v>
       </c>
       <c r="E10" t="n">
-        <v>0.004198</v>
+        <v>0.015001</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H10" t="n">
         <v>24</v>
@@ -715,26 +727,26 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tm_score</t>
+          <t>cavity_frequency_Negatively_charged</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.841</v>
+        <v>0.6032</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8046</v>
+        <v>1.0833</v>
       </c>
       <c r="D11" t="n">
-        <v>3.1394</v>
+        <v>-2.4898</v>
       </c>
       <c r="E11" t="n">
-        <v>0.004229</v>
+        <v>0.018505</v>
       </c>
       <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H11" t="n">
         <v>24</v>
@@ -743,26 +755,26 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>iqr_plddt_bs</t>
+          <t>cavity_volume</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0274</v>
+        <v>512.5644</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0495</v>
+        <v>630.8733</v>
       </c>
       <c r="D12" t="n">
-        <v>-2.9436</v>
+        <v>-2.4129</v>
       </c>
       <c r="E12" t="n">
-        <v>0.006389</v>
+        <v>0.022036</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H12" t="n">
         <v>24</v>
@@ -771,26 +783,26 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cavity_n_points</t>
+          <t>median_plddt_bs</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2395.4821</v>
+        <v>0.9728</v>
       </c>
       <c r="C13" t="n">
-        <v>2925.7083</v>
+        <v>0.9627</v>
       </c>
       <c r="D13" t="n">
-        <v>-2.7743</v>
+        <v>2.2896</v>
       </c>
       <c r="E13" t="n">
-        <v>0.00945</v>
+        <v>0.026323</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H13" t="n">
         <v>24</v>
@@ -799,26 +811,26 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cavity_frequency_Negatively_charged</t>
+          <t>bindingsite_similarity_score</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.5714</v>
+        <v>0.3037</v>
       </c>
       <c r="C14" t="n">
-        <v>1.0833</v>
+        <v>0.2609</v>
       </c>
       <c r="D14" t="n">
-        <v>-2.6467</v>
+        <v>2.3038</v>
       </c>
       <c r="E14" t="n">
-        <v>0.012736</v>
+        <v>0.026744</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H14" t="n">
         <v>24</v>
@@ -827,26 +839,26 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>cavity_volume</t>
+          <t>median_plddt</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>501.4052</v>
+        <v>0.97</v>
       </c>
       <c r="C15" t="n">
-        <v>630.8733</v>
+        <v>0.9597</v>
       </c>
       <c r="D15" t="n">
-        <v>-2.6241</v>
+        <v>2.2676</v>
       </c>
       <c r="E15" t="n">
-        <v>0.013333</v>
+        <v>0.026788</v>
       </c>
       <c r="F15" t="b">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H15" t="n">
         <v>24</v>
@@ -855,26 +867,26 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>iqr_plddt</t>
+          <t>cavity_avg_depth</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.0321</v>
+        <v>1.6106</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0631</v>
+        <v>1.8858</v>
       </c>
       <c r="D16" t="n">
-        <v>-2.6211</v>
+        <v>-2.1798</v>
       </c>
       <c r="E16" t="n">
-        <v>0.014626</v>
+        <v>0.037554</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H16" t="n">
         <v>24</v>
@@ -883,26 +895,26 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>bindingsite_similarity_score</t>
+          <t>n_bindingsite_residues</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.3083</v>
+        <v>43.5556</v>
       </c>
       <c r="C17" t="n">
-        <v>0.2609</v>
+        <v>44.875</v>
       </c>
       <c r="D17" t="n">
-        <v>2.5014</v>
+        <v>-2.1594</v>
       </c>
       <c r="E17" t="n">
-        <v>0.016466</v>
+        <v>0.037561</v>
       </c>
       <c r="F17" t="b">
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H17" t="n">
         <v>24</v>
@@ -911,26 +923,26 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cavity_avg_depth</t>
+          <t>n_res_plddt_bs</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1.5857</v>
+        <v>43.5556</v>
       </c>
       <c r="C18" t="n">
-        <v>1.8858</v>
+        <v>44.875</v>
       </c>
       <c r="D18" t="n">
-        <v>-2.3862</v>
+        <v>-2.1594</v>
       </c>
       <c r="E18" t="n">
-        <v>0.02389</v>
+        <v>0.037561</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H18" t="n">
         <v>24</v>
@@ -939,26 +951,26 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>n_bindingsite_residues</t>
+          <t>cavity_frequency_Alipathic_apolar</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>43.4464</v>
+        <v>9.4444</v>
       </c>
       <c r="C19" t="n">
-        <v>44.875</v>
+        <v>10.9167</v>
       </c>
       <c r="D19" t="n">
-        <v>-2.351</v>
+        <v>-1.9864</v>
       </c>
       <c r="E19" t="n">
-        <v>0.024453</v>
+        <v>0.055386</v>
       </c>
       <c r="F19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H19" t="n">
         <v>24</v>
@@ -967,26 +979,26 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>n_res_plddt_bs</t>
+          <t>iqr_plddt_bs</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>43.4464</v>
+        <v>0.0329</v>
       </c>
       <c r="C20" t="n">
-        <v>44.875</v>
+        <v>0.0495</v>
       </c>
       <c r="D20" t="n">
-        <v>-2.351</v>
+        <v>-1.905</v>
       </c>
       <c r="E20" t="n">
-        <v>0.024453</v>
+        <v>0.06278499999999999</v>
       </c>
       <c r="F20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H20" t="n">
         <v>24</v>
@@ -995,26 +1007,26 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cavity_frequency_Alipathic_apolar</t>
+          <t>iqr_plddt</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>9.321400000000001</v>
+        <v>0.0387</v>
       </c>
       <c r="C21" t="n">
-        <v>10.9167</v>
+        <v>0.0631</v>
       </c>
       <c r="D21" t="n">
-        <v>-2.1191</v>
+        <v>-1.9026</v>
       </c>
       <c r="E21" t="n">
-        <v>0.041325</v>
+        <v>0.065451</v>
       </c>
       <c r="F21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H21" t="n">
         <v>24</v>
@@ -1027,22 +1039,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6.9464</v>
+        <v>7</v>
       </c>
       <c r="C22" t="n">
         <v>7.9167</v>
       </c>
       <c r="D22" t="n">
-        <v>-1.7722</v>
+        <v>-1.6702</v>
       </c>
       <c r="E22" t="n">
-        <v>0.08784400000000001</v>
+        <v>0.106514</v>
       </c>
       <c r="F22" t="b">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H22" t="n">
         <v>24</v>
@@ -1055,22 +1067,22 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2.3393</v>
+        <v>2.3492</v>
       </c>
       <c r="C23" t="n">
         <v>2.7917</v>
       </c>
       <c r="D23" t="n">
-        <v>-1.6244</v>
+        <v>-1.617</v>
       </c>
       <c r="E23" t="n">
-        <v>0.112267</v>
+        <v>0.114311</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H23" t="n">
         <v>24</v>
@@ -1079,26 +1091,26 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cavity_area</t>
+          <t>aligned_fraction</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>364.807</v>
+        <v>0.4657</v>
       </c>
       <c r="C24" t="n">
-        <v>407.1167</v>
+        <v>0.415</v>
       </c>
       <c r="D24" t="n">
-        <v>-1.555</v>
+        <v>1.4418</v>
       </c>
       <c r="E24" t="n">
-        <v>0.128712</v>
+        <v>0.155282</v>
       </c>
       <c r="F24" t="b">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H24" t="n">
         <v>24</v>
@@ -1107,26 +1119,26 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>aligned_fraction</t>
+          <t>cavity_area</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.4643</v>
+        <v>370.1295</v>
       </c>
       <c r="C25" t="n">
-        <v>0.415</v>
+        <v>407.1167</v>
       </c>
       <c r="D25" t="n">
-        <v>1.3586</v>
+        <v>-1.3743</v>
       </c>
       <c r="E25" t="n">
-        <v>0.179741</v>
+        <v>0.178164</v>
       </c>
       <c r="F25" t="b">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H25" t="n">
         <v>24</v>
@@ -1135,26 +1147,26 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>cavity_avg_hydropathy</t>
+          <t>n_aligned_residues</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-0.2739</v>
+        <v>20.3492</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.2275</v>
+        <v>18.5417</v>
       </c>
       <c r="D26" t="n">
-        <v>-1.3032</v>
+        <v>1.1596</v>
       </c>
       <c r="E26" t="n">
-        <v>0.198866</v>
+        <v>0.251276</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H26" t="n">
         <v>24</v>
@@ -1167,22 +1179,22 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.6734</v>
+        <v>0.6693</v>
       </c>
       <c r="C27" t="n">
         <v>0.6228</v>
       </c>
       <c r="D27" t="n">
-        <v>1.1813</v>
+        <v>1.1236</v>
       </c>
       <c r="E27" t="n">
-        <v>0.242348</v>
+        <v>0.266156</v>
       </c>
       <c r="F27" t="b">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H27" t="n">
         <v>24</v>
@@ -1191,26 +1203,26 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>n_aligned_residues</t>
+          <t>rmsd</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>20.2321</v>
+        <v>2.7751</v>
       </c>
       <c r="C28" t="n">
-        <v>18.5417</v>
+        <v>2.7229</v>
       </c>
       <c r="D28" t="n">
-        <v>1.0531</v>
+        <v>1.096</v>
       </c>
       <c r="E28" t="n">
-        <v>0.296731</v>
+        <v>0.280782</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H28" t="n">
         <v>24</v>
@@ -1219,26 +1231,26 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>rmsd</t>
+          <t>cavity_avg_hydropathy</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2.7679</v>
+        <v>-0.2638</v>
       </c>
       <c r="C29" t="n">
-        <v>2.7229</v>
+        <v>-0.2275</v>
       </c>
       <c r="D29" t="n">
-        <v>0.9412</v>
+        <v>-1.0309</v>
       </c>
       <c r="E29" t="n">
-        <v>0.353201</v>
+        <v>0.307986</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H29" t="n">
         <v>24</v>
@@ -1251,22 +1263,22 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>387.875</v>
+        <v>387.5238</v>
       </c>
       <c r="C30" t="n">
         <v>395.125</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.9419</v>
+        <v>-0.9857</v>
       </c>
       <c r="E30" t="n">
-        <v>0.355355</v>
+        <v>0.333738</v>
       </c>
       <c r="F30" t="b">
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H30" t="n">
         <v>24</v>
@@ -1279,22 +1291,22 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7.875</v>
+        <v>7.9365</v>
       </c>
       <c r="C31" t="n">
         <v>8.291700000000001</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.7947</v>
+        <v>-0.6865</v>
       </c>
       <c r="E31" t="n">
-        <v>0.43182</v>
+        <v>0.496807</v>
       </c>
       <c r="F31" t="b">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H31" t="n">
         <v>24</v>
@@ -1303,26 +1315,26 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sequence_identity</t>
+          <t>cavity_rmsd</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.2828</v>
+        <v>0.4987</v>
       </c>
       <c r="C32" t="n">
-        <v>0.281</v>
+        <v>0.5071</v>
       </c>
       <c r="D32" t="n">
-        <v>0.5083</v>
+        <v>-0.4433</v>
       </c>
       <c r="E32" t="n">
-        <v>0.613478</v>
+        <v>0.660402</v>
       </c>
       <c r="F32" t="b">
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H32" t="n">
         <v>24</v>
@@ -1331,26 +1343,26 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>cavity_rmsd</t>
+          <t>sequence_identity</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.4988</v>
+        <v>0.2807</v>
       </c>
       <c r="C33" t="n">
-        <v>0.5071</v>
+        <v>0.281</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.4375</v>
+        <v>-0.1016</v>
       </c>
       <c r="E33" t="n">
-        <v>0.664526</v>
+        <v>0.91945</v>
       </c>
       <c r="F33" t="b">
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H33" t="n">
         <v>24</v>
@@ -1374,7 +1386,7 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="H34" t="n">
         <v>24</v>
@@ -1395,57 +1407,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>column</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>group</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>mean</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>median</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>std</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>var</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>max</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>skewness</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>kurtosis</t>
         </is>
@@ -1463,19 +1475,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4643</v>
+        <v>0.4657</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4939</v>
+        <v>0.4878</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1757</v>
+        <v>0.1721</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0309</v>
+        <v>0.0296</v>
       </c>
       <c r="H2" t="n">
         <v>0.1136</v>
@@ -1484,10 +1496,10 @@
         <v>0.7674</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.1988</v>
+        <v>-0.2</v>
       </c>
       <c r="K2" t="n">
-        <v>-1.1322</v>
+        <v>-1.103</v>
       </c>
     </row>
     <row r="3">
@@ -1541,31 +1553,31 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9549</v>
+        <v>0.95</v>
       </c>
       <c r="E4" t="n">
         <v>0.958</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0185</v>
+        <v>0.0327</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0003</v>
+        <v>0.0011</v>
       </c>
       <c r="H4" t="n">
-        <v>0.865</v>
+        <v>0.741</v>
       </c>
       <c r="I4" t="n">
         <v>0.974</v>
       </c>
       <c r="J4" t="n">
-        <v>-3.0452</v>
+        <v>-4.6168</v>
       </c>
       <c r="K4" t="n">
-        <v>11.3315</v>
+        <v>25.2704</v>
       </c>
     </row>
     <row r="5">
@@ -1619,31 +1631,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9623</v>
+        <v>0.9584</v>
       </c>
       <c r="E6" t="n">
         <v>0.968</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0179</v>
+        <v>0.0315</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0003</v>
+        <v>0.001</v>
       </c>
       <c r="H6" t="n">
-        <v>0.91</v>
+        <v>0.757</v>
       </c>
       <c r="I6" t="n">
         <v>0.983</v>
       </c>
       <c r="J6" t="n">
-        <v>-1.365</v>
+        <v>-4.3877</v>
       </c>
       <c r="K6" t="n">
-        <v>1.4039</v>
+        <v>24.6814</v>
       </c>
     </row>
     <row r="7">
@@ -1697,19 +1709,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3083</v>
+        <v>0.3037</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3231</v>
+        <v>0.3144</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0738</v>
+        <v>0.0721</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0055</v>
+        <v>0.0052</v>
       </c>
       <c r="H8" t="n">
         <v>0.1528</v>
@@ -1718,10 +1730,10 @@
         <v>0.4279</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.2564</v>
+        <v>-0.1224</v>
       </c>
       <c r="K8" t="n">
-        <v>-1.0571</v>
+        <v>-1.0779</v>
       </c>
     </row>
     <row r="9">
@@ -1775,19 +1787,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D10" t="n">
-        <v>364.807</v>
+        <v>370.1295</v>
       </c>
       <c r="E10" t="n">
-        <v>389.945</v>
+        <v>392.7</v>
       </c>
       <c r="F10" t="n">
-        <v>93.568</v>
+        <v>94.0324</v>
       </c>
       <c r="G10" t="n">
-        <v>8754.962600000001</v>
+        <v>8842.085499999999</v>
       </c>
       <c r="H10" t="n">
         <v>204.43</v>
@@ -1796,10 +1808,10 @@
         <v>524.59</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.1042</v>
+        <v>-0.1676</v>
       </c>
       <c r="K10" t="n">
-        <v>-1.2699</v>
+        <v>-1.2601</v>
       </c>
     </row>
     <row r="11">
@@ -1853,19 +1865,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D12" t="n">
-        <v>1.5857</v>
+        <v>1.6106</v>
       </c>
       <c r="E12" t="n">
         <v>1.56</v>
       </c>
       <c r="F12" t="n">
-        <v>0.3041</v>
+        <v>0.3342</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0925</v>
+        <v>0.1117</v>
       </c>
       <c r="H12" t="n">
         <v>1.11</v>
@@ -1874,10 +1886,10 @@
         <v>2.63</v>
       </c>
       <c r="J12" t="n">
-        <v>1.0601</v>
+        <v>0.9879</v>
       </c>
       <c r="K12" t="n">
-        <v>1.9104</v>
+        <v>0.9444</v>
       </c>
     </row>
     <row r="13">
@@ -1931,19 +1943,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.2739</v>
+        <v>-0.2638</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.245</v>
+        <v>-0.24</v>
       </c>
       <c r="F14" t="n">
-        <v>0.154</v>
+        <v>0.1577</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0237</v>
+        <v>0.0249</v>
       </c>
       <c r="H14" t="n">
         <v>-0.63</v>
@@ -1952,10 +1964,10 @@
         <v>0.1</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.3582</v>
+        <v>-0.2488</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.1498</v>
+        <v>-0.0546</v>
       </c>
     </row>
     <row r="15">
@@ -2009,19 +2021,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D16" t="n">
-        <v>9.321400000000001</v>
+        <v>9.4444</v>
       </c>
       <c r="E16" t="n">
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>2.4871</v>
+        <v>2.4215</v>
       </c>
       <c r="G16" t="n">
-        <v>6.1857</v>
+        <v>5.8638</v>
       </c>
       <c r="H16" t="n">
         <v>4</v>
@@ -2030,10 +2042,10 @@
         <v>15</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.2861</v>
+        <v>-0.3576</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.4633</v>
+        <v>-0.3432</v>
       </c>
     </row>
     <row r="17">
@@ -2087,19 +2099,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D18" t="n">
-        <v>4.3929</v>
+        <v>4.3651</v>
       </c>
       <c r="E18" t="n">
         <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>0.9278999999999999</v>
+        <v>0.9211</v>
       </c>
       <c r="G18" t="n">
-        <v>0.861</v>
+        <v>0.8484</v>
       </c>
       <c r="H18" t="n">
         <v>3</v>
@@ -2108,10 +2120,10 @@
         <v>7</v>
       </c>
       <c r="J18" t="n">
-        <v>0.7989000000000001</v>
+        <v>0.714</v>
       </c>
       <c r="K18" t="n">
-        <v>0.6991000000000001</v>
+        <v>0.6358</v>
       </c>
     </row>
     <row r="19">
@@ -2165,19 +2177,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D20" t="n">
-        <v>0.5714</v>
+        <v>0.6032</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>0.5345</v>
+        <v>0.5547</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2857</v>
+        <v>0.3077</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -2186,10 +2198,10 @@
         <v>2</v>
       </c>
       <c r="J20" t="n">
-        <v>0.0735</v>
+        <v>0.1572</v>
       </c>
       <c r="K20" t="n">
-        <v>-1.2215</v>
+        <v>-0.9179</v>
       </c>
     </row>
     <row r="21">
@@ -2243,7 +2255,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -2313,19 +2325,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D24" t="n">
-        <v>7.875</v>
+        <v>7.9365</v>
       </c>
       <c r="E24" t="n">
         <v>8</v>
       </c>
       <c r="F24" t="n">
-        <v>1.8787</v>
+        <v>1.874</v>
       </c>
       <c r="G24" t="n">
-        <v>3.5295</v>
+        <v>3.512</v>
       </c>
       <c r="H24" t="n">
         <v>5</v>
@@ -2334,10 +2346,10 @@
         <v>14</v>
       </c>
       <c r="J24" t="n">
-        <v>0.531</v>
+        <v>0.478</v>
       </c>
       <c r="K24" t="n">
-        <v>0.2763</v>
+        <v>0.0586</v>
       </c>
     </row>
     <row r="25">
@@ -2391,19 +2403,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D26" t="n">
-        <v>2.3393</v>
+        <v>2.3492</v>
       </c>
       <c r="E26" t="n">
         <v>3</v>
       </c>
       <c r="F26" t="n">
-        <v>1.0493</v>
+        <v>1.0342</v>
       </c>
       <c r="G26" t="n">
-        <v>1.101</v>
+        <v>1.0696</v>
       </c>
       <c r="H26" t="n">
         <v>1</v>
@@ -2412,10 +2424,10 @@
         <v>4</v>
       </c>
       <c r="J26" t="n">
-        <v>-0.0448</v>
+        <v>-0.0317</v>
       </c>
       <c r="K26" t="n">
-        <v>-1.2855</v>
+        <v>-1.2301</v>
       </c>
     </row>
     <row r="27">
@@ -2469,19 +2481,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D28" t="n">
-        <v>2395.4821</v>
+        <v>2433.3968</v>
       </c>
       <c r="E28" t="n">
-        <v>2348</v>
+        <v>2360</v>
       </c>
       <c r="F28" t="n">
-        <v>507.0948</v>
+        <v>526.2873</v>
       </c>
       <c r="G28" t="n">
-        <v>257145.0906</v>
+        <v>276978.34</v>
       </c>
       <c r="H28" t="n">
         <v>1171</v>
@@ -2490,10 +2502,10 @@
         <v>3768</v>
       </c>
       <c r="J28" t="n">
-        <v>0.5296</v>
+        <v>0.4465</v>
       </c>
       <c r="K28" t="n">
-        <v>0.5587</v>
+        <v>0.1285</v>
       </c>
     </row>
     <row r="29">
@@ -2547,19 +2559,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D30" t="n">
-        <v>0.4988</v>
+        <v>0.4987</v>
       </c>
       <c r="E30" t="n">
-        <v>0.513</v>
+        <v>0.514</v>
       </c>
       <c r="F30" t="n">
-        <v>0.062</v>
+        <v>0.0633</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0038</v>
+        <v>0.004</v>
       </c>
       <c r="H30" t="n">
         <v>0.314</v>
@@ -2568,10 +2580,10 @@
         <v>0.628</v>
       </c>
       <c r="J30" t="n">
-        <v>-1.0032</v>
+        <v>-1.1492</v>
       </c>
       <c r="K30" t="n">
-        <v>1.8057</v>
+        <v>1.8501</v>
       </c>
     </row>
     <row r="31">
@@ -2625,19 +2637,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D32" t="n">
-        <v>501.4052</v>
+        <v>512.5644</v>
       </c>
       <c r="E32" t="n">
-        <v>518.725</v>
+        <v>526.39</v>
       </c>
       <c r="F32" t="n">
-        <v>141.1967</v>
+        <v>143.3047</v>
       </c>
       <c r="G32" t="n">
-        <v>19936.5157</v>
+        <v>20536.2353</v>
       </c>
       <c r="H32" t="n">
         <v>252.94</v>
@@ -2646,10 +2658,10 @@
         <v>827.0599999999999</v>
       </c>
       <c r="J32" t="n">
-        <v>0.2091</v>
+        <v>0.1454</v>
       </c>
       <c r="K32" t="n">
-        <v>-0.6631</v>
+        <v>-0.7452</v>
       </c>
     </row>
     <row r="33">
@@ -2703,31 +2715,31 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D34" t="n">
-        <v>0.0321</v>
+        <v>0.0387</v>
       </c>
       <c r="E34" t="n">
         <v>0.029</v>
       </c>
       <c r="F34" t="n">
-        <v>0.0191</v>
+        <v>0.0447</v>
       </c>
       <c r="G34" t="n">
-        <v>0.0004</v>
+        <v>0.002</v>
       </c>
       <c r="H34" t="n">
         <v>0.015</v>
       </c>
       <c r="I34" t="n">
-        <v>0.121</v>
+        <v>0.352</v>
       </c>
       <c r="J34" t="n">
-        <v>3.035</v>
+        <v>5.7598</v>
       </c>
       <c r="K34" t="n">
-        <v>10.5667</v>
+        <v>36.904</v>
       </c>
     </row>
     <row r="35">
@@ -2781,31 +2793,31 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0274</v>
+        <v>0.0329</v>
       </c>
       <c r="E36" t="n">
         <v>0.021</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0181</v>
+        <v>0.0403</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0003</v>
+        <v>0.0016</v>
       </c>
       <c r="H36" t="n">
         <v>0.006</v>
       </c>
       <c r="I36" t="n">
-        <v>0.076</v>
+        <v>0.312</v>
       </c>
       <c r="J36" t="n">
-        <v>1.2255</v>
+        <v>5.4484</v>
       </c>
       <c r="K36" t="n">
-        <v>0.6902</v>
+        <v>34.8726</v>
       </c>
     </row>
     <row r="37">
@@ -2859,31 +2871,31 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D38" t="n">
-        <v>0.9736</v>
+        <v>0.97</v>
       </c>
       <c r="E38" t="n">
-        <v>0.9765</v>
+        <v>0.976</v>
       </c>
       <c r="F38" t="n">
-        <v>0.0104</v>
+        <v>0.0248</v>
       </c>
       <c r="G38" t="n">
-        <v>0.0001</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="H38" t="n">
-        <v>0.921</v>
+        <v>0.795</v>
       </c>
       <c r="I38" t="n">
         <v>0.984</v>
       </c>
       <c r="J38" t="n">
-        <v>-2.8104</v>
+        <v>-5.855</v>
       </c>
       <c r="K38" t="n">
-        <v>10.6068</v>
+        <v>38.1023</v>
       </c>
     </row>
     <row r="39">
@@ -2937,31 +2949,31 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D40" t="n">
-        <v>0.9757</v>
+        <v>0.9728</v>
       </c>
       <c r="E40" t="n">
-        <v>0.979</v>
+        <v>0.978</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0106</v>
+        <v>0.0208</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0001</v>
+        <v>0.0004</v>
       </c>
       <c r="H40" t="n">
-        <v>0.926</v>
+        <v>0.835</v>
       </c>
       <c r="I40" t="n">
         <v>0.987</v>
       </c>
       <c r="J40" t="n">
-        <v>-2.3206</v>
+        <v>-4.934</v>
       </c>
       <c r="K40" t="n">
-        <v>7.5383</v>
+        <v>28.938</v>
       </c>
     </row>
     <row r="41">
@@ -3015,19 +3027,19 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D42" t="n">
-        <v>20.2321</v>
+        <v>20.3492</v>
       </c>
       <c r="E42" t="n">
         <v>20</v>
       </c>
       <c r="F42" t="n">
-        <v>7.8694</v>
+        <v>7.7712</v>
       </c>
       <c r="G42" t="n">
-        <v>61.9269</v>
+        <v>60.3922</v>
       </c>
       <c r="H42" t="n">
         <v>5</v>
@@ -3036,10 +3048,10 @@
         <v>33</v>
       </c>
       <c r="J42" t="n">
-        <v>-0.1485</v>
+        <v>-0.1358</v>
       </c>
       <c r="K42" t="n">
-        <v>-1.2154</v>
+        <v>-1.2145</v>
       </c>
     </row>
     <row r="43">
@@ -3093,31 +3105,31 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D44" t="n">
-        <v>43.4464</v>
+        <v>43.5556</v>
       </c>
       <c r="E44" t="n">
         <v>44</v>
       </c>
       <c r="F44" t="n">
-        <v>2.0442</v>
+        <v>2.2272</v>
       </c>
       <c r="G44" t="n">
-        <v>4.1789</v>
+        <v>4.9606</v>
       </c>
       <c r="H44" t="n">
         <v>38</v>
       </c>
       <c r="I44" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J44" t="n">
-        <v>-0.4506</v>
+        <v>-0.0477</v>
       </c>
       <c r="K44" t="n">
-        <v>-0.3895</v>
+        <v>0.0953</v>
       </c>
     </row>
     <row r="45">
@@ -3171,19 +3183,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D46" t="n">
-        <v>387.875</v>
+        <v>387.5238</v>
       </c>
       <c r="E46" t="n">
         <v>389</v>
       </c>
       <c r="F46" t="n">
-        <v>11.0323</v>
+        <v>12.2657</v>
       </c>
       <c r="G46" t="n">
-        <v>121.7114</v>
+        <v>150.447</v>
       </c>
       <c r="H46" t="n">
         <v>341</v>
@@ -3192,10 +3204,10 @@
         <v>441</v>
       </c>
       <c r="J46" t="n">
-        <v>0.5772</v>
+        <v>-0.3925</v>
       </c>
       <c r="K46" t="n">
-        <v>13.2662</v>
+        <v>9.944000000000001</v>
       </c>
     </row>
     <row r="47">
@@ -3249,31 +3261,31 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D48" t="n">
-        <v>43.4464</v>
+        <v>43.5556</v>
       </c>
       <c r="E48" t="n">
         <v>44</v>
       </c>
       <c r="F48" t="n">
-        <v>2.0442</v>
+        <v>2.2272</v>
       </c>
       <c r="G48" t="n">
-        <v>4.1789</v>
+        <v>4.9606</v>
       </c>
       <c r="H48" t="n">
         <v>38</v>
       </c>
       <c r="I48" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J48" t="n">
-        <v>-0.4506</v>
+        <v>-0.0477</v>
       </c>
       <c r="K48" t="n">
-        <v>-0.3895</v>
+        <v>0.0953</v>
       </c>
     </row>
     <row r="49">
@@ -3327,31 +3339,31 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D50" t="n">
-        <v>6.9464</v>
+        <v>7</v>
       </c>
       <c r="E50" t="n">
         <v>7</v>
       </c>
       <c r="F50" t="n">
-        <v>1.0858</v>
+        <v>1.1914</v>
       </c>
       <c r="G50" t="n">
-        <v>1.1789</v>
+        <v>1.4194</v>
       </c>
       <c r="H50" t="n">
         <v>5</v>
       </c>
       <c r="I50" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J50" t="n">
-        <v>-0.1515</v>
+        <v>0.3461</v>
       </c>
       <c r="K50" t="n">
-        <v>-0.7407</v>
+        <v>0.6446</v>
       </c>
     </row>
     <row r="51">
@@ -3405,31 +3417,31 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D52" t="n">
-        <v>0.9039</v>
+        <v>0.8934</v>
       </c>
       <c r="E52" t="n">
-        <v>0.916</v>
+        <v>0.911</v>
       </c>
       <c r="F52" t="n">
-        <v>0.0551</v>
+        <v>0.0788</v>
       </c>
       <c r="G52" t="n">
-        <v>0.003</v>
+        <v>0.0062</v>
       </c>
       <c r="H52" t="n">
-        <v>0.61</v>
+        <v>0.452</v>
       </c>
       <c r="I52" t="n">
         <v>0.952</v>
       </c>
       <c r="J52" t="n">
-        <v>-3.6772</v>
+        <v>-3.8493</v>
       </c>
       <c r="K52" t="n">
-        <v>15.5928</v>
+        <v>16.6382</v>
       </c>
     </row>
     <row r="53">
@@ -3483,31 +3495,31 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D54" t="n">
-        <v>0.9222</v>
+        <v>0.9126</v>
       </c>
       <c r="E54" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F54" t="n">
-        <v>0.0424</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="G54" t="n">
-        <v>0.0018</v>
+        <v>0.0057</v>
       </c>
       <c r="H54" t="n">
-        <v>0.796</v>
+        <v>0.434</v>
       </c>
       <c r="I54" t="n">
         <v>0.973</v>
       </c>
       <c r="J54" t="n">
-        <v>-1.0844</v>
+        <v>-4.2899</v>
       </c>
       <c r="K54" t="n">
-        <v>0.5364</v>
+        <v>24.0946</v>
       </c>
     </row>
     <row r="55">
@@ -3561,19 +3573,19 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D56" t="n">
-        <v>2.7679</v>
+        <v>2.7751</v>
       </c>
       <c r="E56" t="n">
         <v>2.74</v>
       </c>
       <c r="F56" t="n">
-        <v>0.1561</v>
+        <v>0.1628</v>
       </c>
       <c r="G56" t="n">
-        <v>0.0244</v>
+        <v>0.0265</v>
       </c>
       <c r="H56" t="n">
         <v>2.36</v>
@@ -3582,10 +3594,10 @@
         <v>3.22</v>
       </c>
       <c r="J56" t="n">
-        <v>0.341</v>
+        <v>0.2522</v>
       </c>
       <c r="K56" t="n">
-        <v>1.1275</v>
+        <v>0.6229</v>
       </c>
     </row>
     <row r="57">
@@ -3639,19 +3651,19 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D58" t="n">
-        <v>0.6734</v>
+        <v>0.6693</v>
       </c>
       <c r="E58" t="n">
-        <v>0.6457000000000001</v>
+        <v>0.6483</v>
       </c>
       <c r="F58" t="n">
-        <v>0.2114</v>
+        <v>0.2057</v>
       </c>
       <c r="G58" t="n">
-        <v>0.0447</v>
+        <v>0.0423</v>
       </c>
       <c r="H58" t="n">
         <v>0.1404</v>
@@ -3660,10 +3672,10 @@
         <v>1.1226</v>
       </c>
       <c r="J58" t="n">
-        <v>-0.0601</v>
+        <v>-0.0578</v>
       </c>
       <c r="K58" t="n">
-        <v>-0.4851</v>
+        <v>-0.4247</v>
       </c>
     </row>
     <row r="59">
@@ -3717,16 +3729,16 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D60" t="n">
-        <v>0.2828</v>
+        <v>0.2807</v>
       </c>
       <c r="E60" t="n">
-        <v>0.288</v>
+        <v>0.286</v>
       </c>
       <c r="F60" t="n">
-        <v>0.016</v>
+        <v>0.0169</v>
       </c>
       <c r="G60" t="n">
         <v>0.0003</v>
@@ -3738,10 +3750,10 @@
         <v>0.3</v>
       </c>
       <c r="J60" t="n">
-        <v>-1.5342</v>
+        <v>-1.2389</v>
       </c>
       <c r="K60" t="n">
-        <v>3.1235</v>
+        <v>1.7111</v>
       </c>
     </row>
     <row r="61">
@@ -3795,31 +3807,31 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D62" t="n">
-        <v>0.0558</v>
+        <v>0.0599</v>
       </c>
       <c r="E62" t="n">
-        <v>0.0525</v>
+        <v>0.054</v>
       </c>
       <c r="F62" t="n">
-        <v>0.0211</v>
+        <v>0.0272</v>
       </c>
       <c r="G62" t="n">
-        <v>0.0004</v>
+        <v>0.0007</v>
       </c>
       <c r="H62" t="n">
         <v>0.026</v>
       </c>
       <c r="I62" t="n">
-        <v>0.142</v>
+        <v>0.187</v>
       </c>
       <c r="J62" t="n">
-        <v>2.328</v>
+        <v>2.4876</v>
       </c>
       <c r="K62" t="n">
-        <v>7.2819</v>
+        <v>7.7606</v>
       </c>
     </row>
     <row r="63">
@@ -3873,31 +3885,31 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D64" t="n">
-        <v>0.0353</v>
+        <v>0.0381</v>
       </c>
       <c r="E64" t="n">
-        <v>0.0285</v>
+        <v>0.029</v>
       </c>
       <c r="F64" t="n">
-        <v>0.0228</v>
+        <v>0.03</v>
       </c>
       <c r="G64" t="n">
-        <v>0.0005</v>
+        <v>0.0009</v>
       </c>
       <c r="H64" t="n">
-        <v>0.01</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="I64" t="n">
-        <v>0.113</v>
+        <v>0.19</v>
       </c>
       <c r="J64" t="n">
-        <v>1.4131</v>
+        <v>2.5558</v>
       </c>
       <c r="K64" t="n">
-        <v>1.7652</v>
+        <v>9.053599999999999</v>
       </c>
     </row>
     <row r="65">
@@ -3951,19 +3963,19 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D66" t="n">
-        <v>0.841</v>
+        <v>0.8383</v>
       </c>
       <c r="E66" t="n">
-        <v>0.8456</v>
+        <v>0.8454</v>
       </c>
       <c r="F66" t="n">
-        <v>0.02</v>
+        <v>0.0227</v>
       </c>
       <c r="G66" t="n">
-        <v>0.0004</v>
+        <v>0.0005</v>
       </c>
       <c r="H66" t="n">
         <v>0.7452</v>
@@ -3972,10 +3984,10 @@
         <v>0.8761</v>
       </c>
       <c r="J66" t="n">
-        <v>-2.0924</v>
+        <v>-1.807</v>
       </c>
       <c r="K66" t="n">
-        <v>7.6746</v>
+        <v>4.4696</v>
       </c>
     </row>
     <row r="67">
@@ -4032,12 +4044,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
@@ -4060,7 +4072,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4">

</xml_diff>